<commit_message>
add tornado & whirlpool experiments
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
+++ b/ssp_modeling/cost-benefits/cb_config_files/cb_config_params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_morocco/ssp_modeling/cost-benefits/cb_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE71E4E-0326-F648-BF3F-99F95D890A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{957009D5-8AD9-E84A-B1E5-869122919CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="600" windowWidth="51200" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4815" uniqueCount="2069">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4829" uniqueCount="2076">
   <si>
     <t>output_variable_name</t>
   </si>
@@ -6287,6 +6287,27 @@
   </si>
   <si>
     <t>cb:entc:savings_opex:electricity:opex</t>
+  </si>
+  <si>
+    <t>cb:frst:technical_cost:increase_sequestration:X</t>
+  </si>
+  <si>
+    <t>TX:FRST:INCREASE_SEQUESTRATION</t>
+  </si>
+  <si>
+    <t>emission_co2e_co2_frst_sequestration_*</t>
+  </si>
+  <si>
+    <t>$20/ton CO2e additional sequestration</t>
+  </si>
+  <si>
+    <t>Technical cost of increasing forest sequestration</t>
+  </si>
+  <si>
+    <t>Unit cost per additional tCO2e sequestered, applied to the change in emission_co2e_co2_frst_sequestration_* (primary + secondary + mangroves, sum=1) between the strategy and the baseline. Covers management, enrichment planting, fire and grazing control, and monitoring. Area-based drivers are not usable here: the transformation moves the sequestration factor, not the land-use areas.</t>
+  </si>
+  <si>
+    <t>Unit cost of improved forest management / assisted natural regeneration per additional ton of CO2e sequestered (2019 USD). Calibration default; replace with country-specific costs when available.</t>
   </si>
 </sst>
 </file>
@@ -6308,7 +6329,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6324,6 +6345,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6355,7 +6382,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -6363,6 +6390,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6665,7 +6693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E215"/>
+  <dimension ref="A1:E216"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="58.1640625" bestFit="1" customWidth="1"/>
@@ -10317,6 +10345,23 @@
         <v>454</v>
       </c>
       <c r="E215" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A216" t="s">
+        <v>2069</v>
+      </c>
+      <c r="B216" t="s">
+        <v>2073</v>
+      </c>
+      <c r="C216" t="s">
+        <v>2074</v>
+      </c>
+      <c r="D216" t="s">
+        <v>2075</v>
+      </c>
+      <c r="E216" t="s">
         <v>9</v>
       </c>
     </row>
@@ -16822,7 +16867,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L159"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -17364,7 +17408,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>53</v>
       </c>
@@ -17402,7 +17446,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>57</v>
       </c>
@@ -17440,7 +17484,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>62</v>
       </c>
@@ -17478,7 +17522,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>66</v>
       </c>
@@ -17516,7 +17560,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>68</v>
       </c>
@@ -17554,7 +17598,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>70</v>
       </c>
@@ -17592,7 +17636,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -17630,7 +17674,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>74</v>
       </c>
@@ -17668,7 +17712,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>76</v>
       </c>
@@ -17706,7 +17750,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>78</v>
       </c>
@@ -17744,7 +17788,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>80</v>
       </c>
@@ -17782,7 +17826,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>82</v>
       </c>
@@ -17820,7 +17864,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>83</v>
       </c>
@@ -17858,7 +17902,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>85</v>
       </c>
@@ -17896,7 +17940,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>87</v>
       </c>
@@ -17934,7 +17978,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>88</v>
       </c>
@@ -17972,7 +18016,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>90</v>
       </c>
@@ -18010,7 +18054,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>91</v>
       </c>
@@ -18048,7 +18092,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>93</v>
       </c>
@@ -18086,7 +18130,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>95</v>
       </c>
@@ -18124,7 +18168,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>97</v>
       </c>
@@ -18162,7 +18206,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>99</v>
       </c>
@@ -18200,7 +18244,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>100</v>
       </c>
@@ -18238,7 +18282,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>101</v>
       </c>
@@ -18276,7 +18320,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>102</v>
       </c>
@@ -18314,7 +18358,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>103</v>
       </c>
@@ -18352,7 +18396,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>104</v>
       </c>
@@ -18390,7 +18434,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>105</v>
       </c>
@@ -18428,7 +18472,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>106</v>
       </c>
@@ -18466,7 +18510,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>107</v>
       </c>
@@ -18504,7 +18548,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>108</v>
       </c>
@@ -18542,7 +18586,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>109</v>
       </c>
@@ -18580,7 +18624,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>110</v>
       </c>
@@ -18618,7 +18662,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>111</v>
       </c>
@@ -18656,7 +18700,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>112</v>
       </c>
@@ -18694,7 +18738,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>113</v>
       </c>
@@ -18732,7 +18776,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>114</v>
       </c>
@@ -18770,7 +18814,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>115</v>
       </c>
@@ -18808,7 +18852,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>116</v>
       </c>
@@ -18846,7 +18890,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>117</v>
       </c>
@@ -18884,7 +18928,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>118</v>
       </c>
@@ -18922,7 +18966,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>119</v>
       </c>
@@ -18960,7 +19004,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>120</v>
       </c>
@@ -18998,7 +19042,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>121</v>
       </c>
@@ -19036,7 +19080,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>122</v>
       </c>
@@ -19074,7 +19118,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>123</v>
       </c>
@@ -19112,7 +19156,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>124</v>
       </c>
@@ -19150,7 +19194,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>125</v>
       </c>
@@ -19188,7 +19232,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>126</v>
       </c>
@@ -19226,7 +19270,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>127</v>
       </c>
@@ -19264,7 +19308,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>128</v>
       </c>
@@ -19302,7 +19346,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="66" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>131</v>
       </c>
@@ -19340,7 +19384,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="67" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>133</v>
       </c>
@@ -19378,7 +19422,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>135</v>
       </c>
@@ -19416,7 +19460,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>137</v>
       </c>
@@ -19454,7 +19498,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>140</v>
       </c>
@@ -19492,7 +19536,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>151</v>
       </c>
@@ -19530,7 +19574,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>154</v>
       </c>
@@ -19568,7 +19612,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>156</v>
       </c>
@@ -19606,7 +19650,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>158</v>
       </c>
@@ -19644,7 +19688,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>160</v>
       </c>
@@ -19682,7 +19726,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>162</v>
       </c>
@@ -19720,7 +19764,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>164</v>
       </c>
@@ -19758,7 +19802,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>166</v>
       </c>
@@ -19796,7 +19840,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="79" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>184</v>
       </c>
@@ -19834,7 +19878,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>187</v>
       </c>
@@ -19872,7 +19916,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>189</v>
       </c>
@@ -19910,7 +19954,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>206</v>
       </c>
@@ -19948,7 +19992,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>209</v>
       </c>
@@ -19986,7 +20030,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>219</v>
       </c>
@@ -20024,7 +20068,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>232</v>
       </c>
@@ -20062,7 +20106,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>234</v>
       </c>
@@ -20100,7 +20144,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>236</v>
       </c>
@@ -20138,7 +20182,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>238</v>
       </c>
@@ -20176,7 +20220,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>240</v>
       </c>
@@ -20214,7 +20258,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>242</v>
       </c>
@@ -20252,7 +20296,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>244</v>
       </c>
@@ -20290,7 +20334,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>246</v>
       </c>
@@ -20328,7 +20372,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>248</v>
       </c>
@@ -20366,7 +20410,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>262</v>
       </c>
@@ -20404,7 +20448,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>264</v>
       </c>
@@ -20442,7 +20486,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>276</v>
       </c>
@@ -20480,7 +20524,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>279</v>
       </c>
@@ -20518,7 +20562,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>281</v>
       </c>
@@ -20556,7 +20600,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>283</v>
       </c>
@@ -20594,7 +20638,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>284</v>
       </c>
@@ -20632,7 +20676,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>285</v>
       </c>
@@ -20670,7 +20714,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>288</v>
       </c>
@@ -20708,7 +20752,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>290</v>
       </c>
@@ -20746,7 +20790,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>292</v>
       </c>
@@ -20784,7 +20828,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>294</v>
       </c>
@@ -20822,7 +20866,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>297</v>
       </c>
@@ -20860,7 +20904,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>299</v>
       </c>
@@ -20898,7 +20942,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>301</v>
       </c>
@@ -20936,7 +20980,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>303</v>
       </c>
@@ -20974,7 +21018,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>305</v>
       </c>
@@ -21012,7 +21056,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>306</v>
       </c>
@@ -21050,7 +21094,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>309</v>
       </c>
@@ -21088,7 +21132,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>311</v>
       </c>
@@ -21126,7 +21170,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>313</v>
       </c>
@@ -21164,7 +21208,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>315</v>
       </c>
@@ -21202,7 +21246,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>318</v>
       </c>
@@ -21240,7 +21284,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>320</v>
       </c>
@@ -21278,7 +21322,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>322</v>
       </c>
@@ -21316,7 +21360,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>324</v>
       </c>
@@ -21354,7 +21398,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>326</v>
       </c>
@@ -21392,7 +21436,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>354</v>
       </c>
@@ -21430,7 +21474,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>356</v>
       </c>
@@ -21468,7 +21512,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>358</v>
       </c>
@@ -21506,7 +21550,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>362</v>
       </c>
@@ -21544,7 +21588,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="125" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>364</v>
       </c>
@@ -21582,7 +21626,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>366</v>
       </c>
@@ -21620,7 +21664,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>368</v>
       </c>
@@ -21658,7 +21702,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>370</v>
       </c>
@@ -21696,7 +21740,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>372</v>
       </c>
@@ -21734,7 +21778,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>375</v>
       </c>
@@ -21772,7 +21816,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>377</v>
       </c>
@@ -21810,7 +21854,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="132" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>379</v>
       </c>
@@ -21848,7 +21892,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>381</v>
       </c>
@@ -21886,7 +21930,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="134" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>384</v>
       </c>
@@ -21924,7 +21968,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="135" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>387</v>
       </c>
@@ -21962,7 +22006,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="136" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>389</v>
       </c>
@@ -22000,7 +22044,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="137" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>392</v>
       </c>
@@ -22038,7 +22082,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="138" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>394</v>
       </c>
@@ -22076,7 +22120,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="139" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>396</v>
       </c>
@@ -22114,7 +22158,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="140" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>398</v>
       </c>
@@ -22152,7 +22196,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>402</v>
       </c>
@@ -22190,7 +22234,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="142" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>405</v>
       </c>
@@ -22228,7 +22272,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="143" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>408</v>
       </c>
@@ -22266,7 +22310,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="144" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>414</v>
       </c>
@@ -22304,7 +22348,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="145" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>417</v>
       </c>
@@ -22342,7 +22386,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="146" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>419</v>
       </c>
@@ -22380,7 +22424,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="147" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>421</v>
       </c>
@@ -22418,7 +22462,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="148" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>423</v>
       </c>
@@ -22456,7 +22500,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="149" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>425</v>
       </c>
@@ -22494,7 +22538,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="150" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>427</v>
       </c>
@@ -22532,7 +22576,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="151" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>430</v>
       </c>
@@ -22570,7 +22614,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="152" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>432</v>
       </c>
@@ -22608,7 +22652,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="153" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>434</v>
       </c>
@@ -22646,7 +22690,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="154" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>436</v>
       </c>
@@ -22684,7 +22728,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="155" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>438</v>
       </c>
@@ -22722,7 +22766,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="156" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>440</v>
       </c>
@@ -22760,7 +22804,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="157" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>441</v>
       </c>
@@ -22798,7 +22842,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="158" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>443</v>
       </c>
@@ -22836,7 +22880,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="159" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>445</v>
       </c>
@@ -22875,32 +22919,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L159" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="cb:agrc:crop_value:crops_produced:bevs_and_spices"/>
-        <filter val="cb:agrc:crop_value:crops_produced:cereals"/>
-        <filter val="cb:agrc:crop_value:crops_produced:fibers"/>
-        <filter val="cb:agrc:crop_value:crops_produced:fruits"/>
-        <filter val="cb:agrc:crop_value:crops_produced:herbs"/>
-        <filter val="cb:agrc:crop_value:crops_produced:nuts"/>
-        <filter val="cb:agrc:crop_value:crops_produced:other_annual"/>
-        <filter val="cb:agrc:crop_value:crops_produced:other_woody_perennial"/>
-        <filter val="cb:agrc:crop_value:crops_produced:pulses"/>
-        <filter val="cb:agrc:crop_value:crops_produced:rice"/>
-        <filter val="cb:agrc:crop_value:crops_produced:sugar_cane"/>
-        <filter val="cb:agrc:crop_value:crops_produced:tubers"/>
-        <filter val="cb:agrc:crop_value:crops_produced:vegetables"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L159" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.6640625" customWidth="1"/>
@@ -25547,6 +25573,53 @@
         <v>2067</v>
       </c>
     </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A57" s="5" t="s">
+        <v>2069</v>
+      </c>
+      <c r="B57" t="s">
+        <v>2070</v>
+      </c>
+      <c r="C57" t="b">
+        <v>1</v>
+      </c>
+      <c r="D57">
+        <v>99</v>
+      </c>
+      <c r="E57" t="s">
+        <v>7</v>
+      </c>
+      <c r="F57" t="s">
+        <v>7</v>
+      </c>
+      <c r="G57" t="s">
+        <v>744</v>
+      </c>
+      <c r="H57" t="s">
+        <v>2071</v>
+      </c>
+      <c r="I57">
+        <v>20000000</v>
+      </c>
+      <c r="J57" t="s">
+        <v>777</v>
+      </c>
+      <c r="K57">
+        <v>1</v>
+      </c>
+      <c r="L57" t="s">
+        <v>7</v>
+      </c>
+      <c r="M57">
+        <v>99</v>
+      </c>
+      <c r="N57" t="b">
+        <v>1</v>
+      </c>
+      <c r="O57" t="s">
+        <v>2072</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O56" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>